<commit_message>
test(editors): update smoke xlsx specs for cases 2,6,7
</commit_message>
<xml_diff>
--- a/products/Editors/scenarios/smoke/2. Главное окно редактора.xlsx
+++ b/products/Editors/scenarios/smoke/2. Главное окно редактора.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Testing\products\Editors\scenarios\smoke\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBDA4D86-3B8A-4528-85A4-9E4697AF5454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA28740C-689C-4D4D-ABAA-5DCC53A59D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="26">
   <si>
     <t>Расположение</t>
   </si>
@@ -61,12 +61,6 @@
   </si>
   <si>
     <t>smoke</t>
-  </si>
-  <si>
-    <t>Установка и обновление</t>
-  </si>
-  <si>
-    <t>Успешно пройдены</t>
   </si>
   <si>
     <t>Выполнен запуск редактора</t>
@@ -549,17 +543,11 @@
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>8</v>
@@ -573,7 +561,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>8</v>
@@ -582,7 +570,7 @@
         <v>8</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>8</v>
@@ -599,13 +587,13 @@
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>8</v>
@@ -622,13 +610,13 @@
         <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>8</v>
@@ -645,13 +633,13 @@
         <v>8</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>8</v>
@@ -668,13 +656,13 @@
         <v>8</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>8</v>
@@ -691,13 +679,13 @@
         <v>8</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>8</v>
@@ -714,13 +702,13 @@
         <v>8</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>8</v>
@@ -737,13 +725,13 @@
         <v>8</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>8</v>
@@ -751,7 +739,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="E12" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>